<commit_message>
Fix teacher adviser import assignment
</commit_message>
<xml_diff>
--- a/public/templates/teacher_import_template.xlsx
+++ b/public/templates/teacher_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="74">
   <si>
     <r>
       <rPr>
@@ -39,7 +39,7 @@
         <color rgb="FFFFFFFF"/>
         <sz val="11"/>
       </rPr>
-      <t xml:space="preserve">Name
+      <t xml:space="preserve">Teacher/Adviser Name
 </t>
     </r>
     <r>
@@ -125,6 +125,25 @@
         <sz val="9"/>
       </rPr>
       <t>(09XXXXXXXXX)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Email
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="9"/>
+      </rPr>
+      <t>(optional)</t>
     </r>
   </si>
   <si>
@@ -726,18 +745,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -755,6 +775,9 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="3:4" x14ac:dyDescent="0.25"/>
@@ -884,464 +907,464 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
       <c r="G1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" t="s">
-        <v>27</v>
-      </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
         <v>33</v>
       </c>
-      <c r="D6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>32</v>
-      </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s">
         <v>37</v>
       </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
         <v>43</v>
       </c>
-      <c r="D9" t="s">
-        <v>42</v>
-      </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" t="s">
         <v>46</v>
       </c>
-      <c r="D10" t="s">
-        <v>45</v>
-      </c>
       <c r="E10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>